<commit_message>
Add L inf of GSA for FMM
</commit_message>
<xml_diff>
--- a/results/GSA/GSA_FMM.xlsx
+++ b/results/GSA/GSA_FMM.xlsx
@@ -8,13 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://michiganstate-my.sharepoint.com/personal/khoshne1_msu_edu/Documents/PhD/Research/2-SensitivityAnalysis/GSA-SALib/SALib-Results-FMM-FMG/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1834" documentId="8_{7FC6161D-F4CD-0943-AB94-C895F4D8422D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6678B182-452B-F04B-8670-82E25B00C584}"/>
+  <xr:revisionPtr revIDLastSave="1838" documentId="8_{7FC6161D-F4CD-0943-AB94-C895F4D8422D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A0D95FAC-EF4C-5C42-8A2F-7C8C34C3A718}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{2B153E34-0161-5541-A84A-F5872730D56D}"/>
   </bookViews>
   <sheets>
-    <sheet name="Storage &amp; Loss Modules" sheetId="3" r:id="rId1"/>
-    <sheet name="Complex Module" sheetId="4" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="3" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="17">
   <si>
     <t>20HS</t>
   </si>
@@ -112,7 +111,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -131,12 +130,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -150,7 +143,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -183,9 +176,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -545,39 +535,39 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
-      <c r="K2" s="14" t="s">
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13"/>
+      <c r="I2" s="13"/>
+      <c r="K2" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="L2" s="14"/>
-      <c r="M2" s="14"/>
-      <c r="N2" s="14"/>
-      <c r="O2" s="14"/>
-      <c r="P2" s="14"/>
-      <c r="Q2" s="14"/>
-      <c r="R2" s="14"/>
-      <c r="S2" s="14"/>
-      <c r="U2" s="14" t="s">
+      <c r="L2" s="13"/>
+      <c r="M2" s="13"/>
+      <c r="N2" s="13"/>
+      <c r="O2" s="13"/>
+      <c r="P2" s="13"/>
+      <c r="Q2" s="13"/>
+      <c r="R2" s="13"/>
+      <c r="S2" s="13"/>
+      <c r="U2" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="V2" s="14"/>
-      <c r="W2" s="14"/>
-      <c r="X2" s="14"/>
-      <c r="Y2" s="14"/>
-      <c r="Z2" s="14"/>
-      <c r="AA2" s="14"/>
-      <c r="AB2" s="14"/>
-      <c r="AC2" s="14"/>
+      <c r="V2" s="13"/>
+      <c r="W2" s="13"/>
+      <c r="X2" s="13"/>
+      <c r="Y2" s="13"/>
+      <c r="Z2" s="13"/>
+      <c r="AA2" s="13"/>
+      <c r="AB2" s="13"/>
+      <c r="AC2" s="13"/>
     </row>
     <row r="3" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
@@ -663,7 +653,7 @@
       </c>
     </row>
     <row r="4" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="12" t="s">
         <v>0</v>
       </c>
       <c r="B4" s="5">
@@ -690,7 +680,7 @@
       <c r="I4" s="2">
         <v>0.71260926163508698</v>
       </c>
-      <c r="K4" s="13" t="s">
+      <c r="K4" s="12" t="s">
         <v>0</v>
       </c>
       <c r="L4" s="5">
@@ -717,7 +707,7 @@
       <c r="S4" s="4">
         <v>5.8056203992543798E-2</v>
       </c>
-      <c r="U4" s="13" t="s">
+      <c r="U4" s="12" t="s">
         <v>0</v>
       </c>
       <c r="V4" s="5">
@@ -746,7 +736,7 @@
       </c>
     </row>
     <row r="5" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A5" s="13"/>
+      <c r="A5" s="12"/>
       <c r="B5" s="7">
         <v>0.5</v>
       </c>
@@ -771,7 +761,7 @@
       <c r="I5" s="8">
         <v>0.62752991157205595</v>
       </c>
-      <c r="K5" s="13"/>
+      <c r="K5" s="12"/>
       <c r="L5" s="7">
         <v>0.5</v>
       </c>
@@ -796,7 +786,7 @@
       <c r="S5" s="11">
         <v>6.4173228857097699E-3</v>
       </c>
-      <c r="U5" s="13"/>
+      <c r="U5" s="12"/>
       <c r="V5" s="7">
         <v>0.5</v>
       </c>
@@ -823,7 +813,7 @@
       </c>
     </row>
     <row r="6" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A6" s="13"/>
+      <c r="A6" s="12"/>
       <c r="B6" s="5">
         <v>1</v>
       </c>
@@ -848,7 +838,7 @@
       <c r="I6" s="2">
         <v>0.72488277830237302</v>
       </c>
-      <c r="K6" s="13"/>
+      <c r="K6" s="12"/>
       <c r="L6" s="5">
         <v>1</v>
       </c>
@@ -873,7 +863,7 @@
       <c r="S6" s="4">
         <v>7.7678435569508597E-2</v>
       </c>
-      <c r="U6" s="13"/>
+      <c r="U6" s="12"/>
       <c r="V6" s="5">
         <v>1</v>
       </c>
@@ -900,7 +890,7 @@
       </c>
     </row>
     <row r="7" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A7" s="13"/>
+      <c r="A7" s="12"/>
       <c r="B7" s="7">
         <v>1.5</v>
       </c>
@@ -925,7 +915,7 @@
       <c r="I7" s="8">
         <v>0.69561742153988204</v>
       </c>
-      <c r="K7" s="13"/>
+      <c r="K7" s="12"/>
       <c r="L7" s="7">
         <v>1.5</v>
       </c>
@@ -950,7 +940,7 @@
       <c r="S7" s="11">
         <v>3.62361043776687E-2</v>
       </c>
-      <c r="U7" s="13"/>
+      <c r="U7" s="12"/>
       <c r="V7" s="7">
         <v>1.5</v>
       </c>
@@ -980,93 +970,93 @@
       <c r="B8" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="15">
+      <c r="C8" s="14">
         <f t="shared" ref="C8:I8" si="0">AVERAGE(C4:C7)</f>
         <v>0.98430394766045226</v>
       </c>
-      <c r="D8" s="15">
+      <c r="D8" s="14">
         <f t="shared" si="0"/>
         <v>9.6561761582580299E-2</v>
       </c>
-      <c r="E8" s="15">
+      <c r="E8" s="14">
         <f t="shared" si="0"/>
         <v>0.89332370245460879</v>
       </c>
-      <c r="F8" s="15">
+      <c r="F8" s="14">
         <f t="shared" ref="F8" si="1">AVERAGE(F4:F7)</f>
         <v>9.5039136561903166E-3</v>
       </c>
-      <c r="G8" s="15">
+      <c r="G8" s="14">
         <f t="shared" si="0"/>
         <v>0.40183809019651473</v>
       </c>
-      <c r="H8" s="15">
+      <c r="H8" s="14">
         <f t="shared" si="0"/>
         <v>2.8277994595202723E-3</v>
       </c>
-      <c r="I8" s="15">
+      <c r="I8" s="14">
         <f t="shared" si="0"/>
         <v>0.69015984326234958</v>
       </c>
       <c r="L8" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="M8" s="15">
+      <c r="M8" s="14">
         <f t="shared" ref="M8:S8" si="2">AVERAGE(M4:M7)</f>
         <v>0.89584042331261826</v>
       </c>
-      <c r="N8" s="15">
+      <c r="N8" s="14">
         <f t="shared" si="2"/>
         <v>0.11552962791568724</v>
       </c>
-      <c r="O8" s="15">
+      <c r="O8" s="14">
         <f t="shared" si="2"/>
         <v>0.92772324836490627</v>
       </c>
-      <c r="P8" s="15">
+      <c r="P8" s="14">
         <f t="shared" ref="P8" si="3">AVERAGE(P4:P7)</f>
         <v>0.12220592859825219</v>
       </c>
-      <c r="Q8" s="15">
+      <c r="Q8" s="14">
         <f t="shared" si="2"/>
         <v>0.53771630779196944</v>
       </c>
-      <c r="R8" s="15">
+      <c r="R8" s="14">
         <f t="shared" si="2"/>
         <v>2.9908017254414573E-3</v>
       </c>
-      <c r="S8" s="15">
+      <c r="S8" s="14">
         <f t="shared" si="2"/>
         <v>4.4597016706357719E-2</v>
       </c>
       <c r="V8" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="W8" s="15">
+      <c r="W8" s="14">
         <f t="shared" ref="W8:AC8" si="4">AVERAGE(W4:W7)</f>
         <v>0.98475318343869911</v>
       </c>
-      <c r="X8" s="15">
+      <c r="X8" s="14">
         <f t="shared" si="4"/>
         <v>9.82906758394438E-2</v>
       </c>
-      <c r="Y8" s="15">
+      <c r="Y8" s="14">
         <f t="shared" si="4"/>
         <v>0.8875651067414807</v>
       </c>
-      <c r="Z8" s="15">
+      <c r="Z8" s="14">
         <f t="shared" si="4"/>
         <v>1.0351439233996434E-2</v>
       </c>
-      <c r="AA8" s="15">
+      <c r="AA8" s="14">
         <f t="shared" si="4"/>
         <v>0.40018392144203252</v>
       </c>
-      <c r="AB8" s="15">
+      <c r="AB8" s="14">
         <f t="shared" si="4"/>
         <v>2.8402579363828E-3</v>
       </c>
-      <c r="AC8" s="15">
+      <c r="AC8" s="14">
         <f t="shared" si="4"/>
         <v>0.68436460776371355</v>
       </c>
@@ -1075,93 +1065,93 @@
       <c r="B9" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="15">
+      <c r="C9" s="14">
         <f>STDEV(C4:C7)</f>
         <v>4.1789461232305657E-3</v>
       </c>
-      <c r="D9" s="15">
+      <c r="D9" s="14">
         <f t="shared" ref="D9:I9" si="5">STDEV(D4:D7)</f>
         <v>4.3681676034632091E-3</v>
       </c>
-      <c r="E9" s="15">
+      <c r="E9" s="14">
         <f t="shared" si="5"/>
         <v>2.0270312727628383E-2</v>
       </c>
-      <c r="F9" s="15">
+      <c r="F9" s="14">
         <f t="shared" ref="F9" si="6">STDEV(F4:F7)</f>
         <v>4.3021623427845586E-3</v>
       </c>
-      <c r="G9" s="15">
+      <c r="G9" s="14">
         <f t="shared" si="5"/>
         <v>3.7784091997727969E-2</v>
       </c>
-      <c r="H9" s="15">
+      <c r="H9" s="14">
         <f t="shared" si="5"/>
         <v>3.8026688067393236E-4</v>
       </c>
-      <c r="I9" s="15">
+      <c r="I9" s="14">
         <f t="shared" si="5"/>
         <v>4.3443266095963697E-2</v>
       </c>
       <c r="L9" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="M9" s="15">
+      <c r="M9" s="14">
         <f>STDEV(M4:M7)</f>
         <v>4.7954524841925788E-3</v>
       </c>
-      <c r="N9" s="15">
+      <c r="N9" s="14">
         <f t="shared" ref="N9:S9" si="7">STDEV(N4:N7)</f>
         <v>4.6851477603288118E-3</v>
       </c>
-      <c r="O9" s="15">
+      <c r="O9" s="14">
         <f t="shared" si="7"/>
         <v>1.3056161296813192E-2</v>
       </c>
-      <c r="P9" s="15">
+      <c r="P9" s="14">
         <f t="shared" ref="P9" si="8">STDEV(P4:P7)</f>
         <v>3.7500752982690934E-2</v>
       </c>
-      <c r="Q9" s="15">
+      <c r="Q9" s="14">
         <f t="shared" si="7"/>
         <v>2.1654157628751732E-2</v>
       </c>
-      <c r="R9" s="15">
+      <c r="R9" s="14">
         <f t="shared" si="7"/>
         <v>7.8984225097161981E-4</v>
       </c>
-      <c r="S9" s="15">
+      <c r="S9" s="14">
         <f t="shared" si="7"/>
         <v>3.0567541999154992E-2</v>
       </c>
       <c r="V9" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="W9" s="15">
+      <c r="W9" s="14">
         <f>STDEV(W4:W7)</f>
         <v>4.1148292902571095E-3</v>
       </c>
-      <c r="X9" s="15">
+      <c r="X9" s="14">
         <f t="shared" ref="X9:AC9" si="9">STDEV(X4:X7)</f>
         <v>4.4350788569674383E-3</v>
       </c>
-      <c r="Y9" s="15">
+      <c r="Y9" s="14">
         <f t="shared" si="9"/>
         <v>2.1242585363527126E-2</v>
       </c>
-      <c r="Z9" s="15">
+      <c r="Z9" s="14">
         <f t="shared" si="9"/>
         <v>4.4967226779570098E-3</v>
       </c>
-      <c r="AA9" s="15">
+      <c r="AA9" s="14">
         <f t="shared" si="9"/>
         <v>3.8192759081880141E-2</v>
       </c>
-      <c r="AB9" s="15">
+      <c r="AB9" s="14">
         <f t="shared" si="9"/>
         <v>3.3239501158298704E-4</v>
       </c>
-      <c r="AC9" s="15">
+      <c r="AC9" s="14">
         <f t="shared" si="9"/>
         <v>4.2016828878300355E-2</v>
       </c>
@@ -1246,7 +1236,7 @@
       </c>
     </row>
     <row r="11" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A11" s="13" t="s">
+      <c r="A11" s="12" t="s">
         <v>7</v>
       </c>
       <c r="B11" s="5">
@@ -1273,7 +1263,7 @@
       <c r="I11" s="4">
         <v>0.33898653849650701</v>
       </c>
-      <c r="K11" s="13" t="s">
+      <c r="K11" s="12" t="s">
         <v>7</v>
       </c>
       <c r="L11" s="5">
@@ -1329,7 +1319,7 @@
       </c>
     </row>
     <row r="12" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A12" s="13"/>
+      <c r="A12" s="12"/>
       <c r="B12" s="7">
         <v>0.5</v>
       </c>
@@ -1354,7 +1344,7 @@
       <c r="I12" s="10">
         <v>0.434015825094482</v>
       </c>
-      <c r="K12" s="13"/>
+      <c r="K12" s="12"/>
       <c r="L12" s="7">
         <v>0.5</v>
       </c>
@@ -1406,7 +1396,7 @@
       </c>
     </row>
     <row r="13" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A13" s="13"/>
+      <c r="A13" s="12"/>
       <c r="B13" s="5">
         <v>1</v>
       </c>
@@ -1431,7 +1421,7 @@
       <c r="I13" s="6">
         <v>0.42509967560708301</v>
       </c>
-      <c r="K13" s="13"/>
+      <c r="K13" s="12"/>
       <c r="L13" s="5">
         <v>1</v>
       </c>
@@ -1483,7 +1473,7 @@
       </c>
     </row>
     <row r="14" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A14" s="13"/>
+      <c r="A14" s="12"/>
       <c r="B14" s="7">
         <v>1.5</v>
       </c>
@@ -1508,7 +1498,7 @@
       <c r="I14" s="10">
         <v>0.57863222638376</v>
       </c>
-      <c r="K14" s="13"/>
+      <c r="K14" s="12"/>
       <c r="L14" s="7">
         <v>1.5</v>
       </c>
@@ -1563,93 +1553,93 @@
       <c r="B15" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C15" s="15">
+      <c r="C15" s="14">
         <f t="shared" ref="C15:I15" si="10">AVERAGE(C11:C14)</f>
         <v>0.96369246383315776</v>
       </c>
-      <c r="D15" s="15">
+      <c r="D15" s="14">
         <f t="shared" si="10"/>
         <v>4.3809317771797376E-2</v>
       </c>
-      <c r="E15" s="15">
+      <c r="E15" s="14">
         <f t="shared" si="10"/>
         <v>0.77497313512424459</v>
       </c>
-      <c r="F15" s="15">
+      <c r="F15" s="14">
         <f t="shared" ref="F15" si="11">AVERAGE(F11:F14)</f>
         <v>1.0841964657394997E-2</v>
       </c>
-      <c r="G15" s="15">
+      <c r="G15" s="14">
         <f t="shared" si="10"/>
         <v>0.49268146121970152</v>
       </c>
-      <c r="H15" s="15">
+      <c r="H15" s="14">
         <f t="shared" si="10"/>
         <v>1.5413325338887074E-3</v>
       </c>
-      <c r="I15" s="15">
+      <c r="I15" s="14">
         <f t="shared" si="10"/>
         <v>0.44418356639545803</v>
       </c>
       <c r="L15" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="M15" s="15">
+      <c r="M15" s="14">
         <f t="shared" ref="M15:S15" si="12">AVERAGE(M11:M14)</f>
         <v>0.94343710655799395</v>
       </c>
-      <c r="N15" s="15">
+      <c r="N15" s="14">
         <f t="shared" si="12"/>
         <v>5.5039688610784197E-2</v>
       </c>
-      <c r="O15" s="15">
+      <c r="O15" s="14">
         <f t="shared" si="12"/>
         <v>0.87228001036056568</v>
       </c>
-      <c r="P15" s="15">
+      <c r="P15" s="14">
         <f t="shared" ref="P15" si="13">AVERAGE(P11:P14)</f>
         <v>0.14316491252324848</v>
       </c>
-      <c r="Q15" s="15">
+      <c r="Q15" s="14">
         <f t="shared" si="12"/>
         <v>0.17252652772809374</v>
       </c>
-      <c r="R15" s="15">
+      <c r="R15" s="14">
         <f t="shared" si="12"/>
         <v>4.0033900157744585E-4</v>
       </c>
-      <c r="S15" s="15">
+      <c r="S15" s="14">
         <f t="shared" si="12"/>
         <v>1.7142185899699625E-2</v>
       </c>
       <c r="V15" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="W15" s="15">
+      <c r="W15" s="14">
         <f t="shared" ref="W15:AC15" si="14">AVERAGE(W11:W14)</f>
         <v>0.96365690374411317</v>
       </c>
-      <c r="X15" s="15">
+      <c r="X15" s="14">
         <f t="shared" si="14"/>
         <v>4.4284643262253301E-2</v>
       </c>
-      <c r="Y15" s="15">
+      <c r="Y15" s="14">
         <f t="shared" si="14"/>
         <v>0.77127992586344785</v>
       </c>
-      <c r="Z15" s="15">
+      <c r="Z15" s="14">
         <f t="shared" si="14"/>
         <v>1.1666424584806039E-2</v>
       </c>
-      <c r="AA15" s="15">
+      <c r="AA15" s="14">
         <f t="shared" si="14"/>
         <v>0.49172214541184828</v>
       </c>
-      <c r="AB15" s="15">
+      <c r="AB15" s="14">
         <f t="shared" si="14"/>
         <v>1.5176593120884E-3</v>
       </c>
-      <c r="AC15" s="15">
+      <c r="AC15" s="14">
         <f t="shared" si="14"/>
         <v>0.4362262800309985</v>
       </c>
@@ -1658,93 +1648,93 @@
       <c r="B16" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C16" s="15">
+      <c r="C16" s="14">
         <f>STDEV(C11:C14)</f>
         <v>1.2952407405550285E-2</v>
       </c>
-      <c r="D16" s="15">
+      <c r="D16" s="14">
         <f t="shared" ref="D16:I16" si="15">STDEV(D11:D14)</f>
         <v>3.5679363612889613E-3</v>
       </c>
-      <c r="E16" s="15">
+      <c r="E16" s="14">
         <f t="shared" si="15"/>
         <v>3.2562984527060058E-2</v>
       </c>
-      <c r="F16" s="15">
+      <c r="F16" s="14">
         <f t="shared" ref="F16" si="16">STDEV(F11:F14)</f>
         <v>1.3005882185945609E-2</v>
       </c>
-      <c r="G16" s="15">
+      <c r="G16" s="14">
         <f t="shared" si="15"/>
         <v>5.3475270181742626E-2</v>
       </c>
-      <c r="H16" s="15">
+      <c r="H16" s="14">
         <f t="shared" si="15"/>
         <v>5.072884254373692E-4</v>
       </c>
-      <c r="I16" s="15">
+      <c r="I16" s="14">
         <f t="shared" si="15"/>
         <v>9.9348602912855646E-2</v>
       </c>
       <c r="L16" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="M16" s="15">
+      <c r="M16" s="14">
         <f>STDEV(M11:M14)</f>
         <v>9.3256974439924097E-3</v>
       </c>
-      <c r="N16" s="15">
+      <c r="N16" s="14">
         <f t="shared" ref="N16:S16" si="17">STDEV(N11:N14)</f>
         <v>4.9864535293932463E-3</v>
       </c>
-      <c r="O16" s="15">
+      <c r="O16" s="14">
         <f t="shared" si="17"/>
         <v>2.2420372307615091E-2</v>
       </c>
-      <c r="P16" s="15">
+      <c r="P16" s="14">
         <f t="shared" ref="P16" si="18">STDEV(P11:P14)</f>
         <v>0.14924445349198986</v>
       </c>
-      <c r="Q16" s="15">
+      <c r="Q16" s="14">
         <f t="shared" si="17"/>
         <v>9.7775717260037878E-2</v>
       </c>
-      <c r="R16" s="15">
+      <c r="R16" s="14">
         <f t="shared" si="17"/>
         <v>4.6466243173908585E-4</v>
       </c>
-      <c r="S16" s="15">
+      <c r="S16" s="14">
         <f t="shared" si="17"/>
         <v>5.9019257921697236E-3</v>
       </c>
       <c r="V16" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="W16" s="15">
+      <c r="W16" s="14">
         <f>STDEV(W11:W14)</f>
         <v>1.3432603043800383E-2</v>
       </c>
-      <c r="X16" s="15">
+      <c r="X16" s="14">
         <f t="shared" ref="X16:AC16" si="19">STDEV(X11:X14)</f>
         <v>3.7410496009907287E-3</v>
       </c>
-      <c r="Y16" s="15">
+      <c r="Y16" s="14">
         <f t="shared" si="19"/>
         <v>3.339227786399826E-2</v>
       </c>
-      <c r="Z16" s="15">
+      <c r="Z16" s="14">
         <f t="shared" si="19"/>
         <v>1.4010696265650055E-2</v>
       </c>
-      <c r="AA16" s="15">
+      <c r="AA16" s="14">
         <f t="shared" si="19"/>
         <v>5.3850940532158602E-2</v>
       </c>
-      <c r="AB16" s="15">
+      <c r="AB16" s="14">
         <f t="shared" si="19"/>
         <v>4.6194936313897729E-4</v>
       </c>
-      <c r="AC16" s="15">
+      <c r="AC16" s="14">
         <f t="shared" si="19"/>
         <v>9.8976840210903888E-2</v>
       </c>
@@ -1829,7 +1819,7 @@
       </c>
     </row>
     <row r="18" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A18" s="13" t="s">
+      <c r="A18" s="12" t="s">
         <v>8</v>
       </c>
       <c r="B18" s="5">
@@ -1856,7 +1846,7 @@
       <c r="I18" s="4">
         <v>0.25150224598864801</v>
       </c>
-      <c r="K18" s="13" t="s">
+      <c r="K18" s="12" t="s">
         <v>8</v>
       </c>
       <c r="L18" s="5">
@@ -1883,7 +1873,7 @@
       <c r="S18" s="4">
         <v>5.9823732703551402E-2</v>
       </c>
-      <c r="U18" s="13" t="s">
+      <c r="U18" s="12" t="s">
         <v>8</v>
       </c>
       <c r="V18" s="5">
@@ -1912,7 +1902,7 @@
       </c>
     </row>
     <row r="19" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A19" s="13"/>
+      <c r="A19" s="12"/>
       <c r="B19" s="7">
         <v>0.5</v>
       </c>
@@ -1937,7 +1927,7 @@
       <c r="I19" s="11">
         <v>0.18400288481664101</v>
       </c>
-      <c r="K19" s="13"/>
+      <c r="K19" s="12"/>
       <c r="L19" s="7">
         <v>0.5</v>
       </c>
@@ -1962,7 +1952,7 @@
       <c r="S19" s="11">
         <v>3.9973829435990503E-2</v>
       </c>
-      <c r="U19" s="13"/>
+      <c r="U19" s="12"/>
       <c r="V19" s="7">
         <v>0.5</v>
       </c>
@@ -1989,7 +1979,7 @@
       </c>
     </row>
     <row r="20" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A20" s="13"/>
+      <c r="A20" s="12"/>
       <c r="B20" s="5">
         <v>1</v>
       </c>
@@ -2014,7 +2004,7 @@
       <c r="I20" s="4">
         <v>0.27923909196614199</v>
       </c>
-      <c r="K20" s="13"/>
+      <c r="K20" s="12"/>
       <c r="L20" s="5">
         <v>1</v>
       </c>
@@ -2039,7 +2029,7 @@
       <c r="S20" s="4">
         <v>4.1678811158526403E-2</v>
       </c>
-      <c r="U20" s="13"/>
+      <c r="U20" s="12"/>
       <c r="V20" s="5">
         <v>1</v>
       </c>
@@ -2066,7 +2056,7 @@
       </c>
     </row>
     <row r="21" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A21" s="13"/>
+      <c r="A21" s="12"/>
       <c r="B21" s="7">
         <v>1.5</v>
       </c>
@@ -2091,7 +2081,7 @@
       <c r="I21" s="11">
         <v>0.209353811184638</v>
       </c>
-      <c r="K21" s="13"/>
+      <c r="K21" s="12"/>
       <c r="L21" s="7">
         <v>1.5</v>
       </c>
@@ -2116,7 +2106,7 @@
       <c r="S21" s="11">
         <v>6.5759896618660996E-2</v>
       </c>
-      <c r="U21" s="13"/>
+      <c r="U21" s="12"/>
       <c r="V21" s="7">
         <v>1.5</v>
       </c>
@@ -2146,93 +2136,93 @@
       <c r="B22" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C22" s="15">
+      <c r="C22" s="14">
         <f t="shared" ref="C22:I22" si="20">AVERAGE(C18:C21)</f>
         <v>0.92295158060746996</v>
       </c>
-      <c r="D22" s="15">
+      <c r="D22" s="14">
         <f t="shared" si="20"/>
         <v>2.4777611168569101E-2</v>
       </c>
-      <c r="E22" s="15">
+      <c r="E22" s="14">
         <f t="shared" si="20"/>
         <v>0.58750819310499947</v>
       </c>
-      <c r="F22" s="15">
+      <c r="F22" s="14">
         <f t="shared" ref="F22" si="21">AVERAGE(F18:F21)</f>
         <v>7.0542024279367978E-3</v>
       </c>
-      <c r="G22" s="15">
+      <c r="G22" s="14">
         <f t="shared" si="20"/>
         <v>0.66497579375516958</v>
       </c>
-      <c r="H22" s="15">
+      <c r="H22" s="14">
         <f t="shared" si="20"/>
         <v>7.7485682680579883E-4</v>
       </c>
-      <c r="I22" s="15">
+      <c r="I22" s="14">
         <f t="shared" si="20"/>
         <v>0.23102450848901726</v>
       </c>
       <c r="L22" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="M22" s="15">
+      <c r="M22" s="14">
         <f t="shared" ref="M22:S22" si="22">AVERAGE(M18:M21)</f>
         <v>0.95031053239881969</v>
       </c>
-      <c r="N22" s="15">
+      <c r="N22" s="14">
         <f t="shared" si="22"/>
         <v>3.4630708761829679E-2</v>
       </c>
-      <c r="O22" s="15">
+      <c r="O22" s="14">
         <f t="shared" ref="O22:P22" si="23">AVERAGE(O18:O21)</f>
         <v>0.79637887608683622</v>
       </c>
-      <c r="P22" s="15">
+      <c r="P22" s="14">
         <f t="shared" si="23"/>
         <v>8.5599464518052823E-2</v>
       </c>
-      <c r="Q22" s="15">
+      <c r="Q22" s="14">
         <f t="shared" si="22"/>
         <v>0.12282378005753801</v>
       </c>
-      <c r="R22" s="15">
+      <c r="R22" s="14">
         <f t="shared" si="22"/>
         <v>3.6149830059286133E-5</v>
       </c>
-      <c r="S22" s="15">
+      <c r="S22" s="14">
         <f t="shared" si="22"/>
         <v>5.1809067479182326E-2</v>
       </c>
       <c r="V22" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="W22" s="15">
+      <c r="W22" s="14">
         <f t="shared" ref="W22:AC22" si="24">AVERAGE(W18:W21)</f>
         <v>0.92316638219374203</v>
       </c>
-      <c r="X22" s="15">
+      <c r="X22" s="14">
         <f t="shared" si="24"/>
         <v>2.5041813041231504E-2</v>
       </c>
-      <c r="Y22" s="15">
+      <c r="Y22" s="14">
         <f t="shared" si="24"/>
         <v>0.58526151618597022</v>
       </c>
-      <c r="Z22" s="15">
+      <c r="Z22" s="14">
         <f t="shared" si="24"/>
         <v>7.4651319864325544E-3</v>
       </c>
-      <c r="AA22" s="15">
+      <c r="AA22" s="14">
         <f t="shared" si="24"/>
         <v>0.66386991787808447</v>
       </c>
-      <c r="AB22" s="15">
+      <c r="AB22" s="14">
         <f t="shared" si="24"/>
         <v>7.665486163292998E-4</v>
       </c>
-      <c r="AC22" s="15">
+      <c r="AC22" s="14">
         <f t="shared" si="24"/>
         <v>0.22701088471674125</v>
       </c>
@@ -2241,93 +2231,93 @@
       <c r="B23" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C23" s="15">
+      <c r="C23" s="14">
         <f>STDEV(C18:C21)</f>
         <v>1.7293191314849535E-2</v>
       </c>
-      <c r="D23" s="15">
+      <c r="D23" s="14">
         <f t="shared" ref="D23:I23" si="25">STDEV(D18:D21)</f>
         <v>1.4052906796232249E-3</v>
       </c>
-      <c r="E23" s="15">
+      <c r="E23" s="14">
         <f t="shared" si="25"/>
         <v>5.3585431119679623E-2</v>
       </c>
-      <c r="F23" s="15">
+      <c r="F23" s="14">
         <f t="shared" ref="F23" si="26">STDEV(F18:F21)</f>
         <v>1.1563709616679047E-2</v>
       </c>
-      <c r="G23" s="15">
+      <c r="G23" s="14">
         <f t="shared" si="25"/>
         <v>4.5458222257335715E-2</v>
       </c>
-      <c r="H23" s="15">
+      <c r="H23" s="14">
         <f t="shared" si="25"/>
         <v>1.6588609959457902E-4</v>
       </c>
-      <c r="I23" s="15">
+      <c r="I23" s="14">
         <f t="shared" si="25"/>
         <v>4.2523076117252659E-2</v>
       </c>
       <c r="L23" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="M23" s="15">
+      <c r="M23" s="14">
         <f>STDEV(M18:M21)</f>
         <v>7.1601353362398933E-3</v>
       </c>
-      <c r="N23" s="15">
+      <c r="N23" s="14">
         <f t="shared" ref="N23:S23" si="27">STDEV(N18:N21)</f>
         <v>2.1357469021107919E-3</v>
       </c>
-      <c r="O23" s="15">
+      <c r="O23" s="14">
         <f t="shared" ref="O23:P23" si="28">STDEV(O18:O21)</f>
         <v>2.8074360339986754E-2</v>
       </c>
-      <c r="P23" s="15">
+      <c r="P23" s="14">
         <f t="shared" si="28"/>
         <v>0.11446294816503529</v>
       </c>
-      <c r="Q23" s="15">
+      <c r="Q23" s="14">
         <f t="shared" si="27"/>
         <v>3.0303133467503744E-2</v>
       </c>
-      <c r="R23" s="15">
+      <c r="R23" s="14">
         <f t="shared" si="27"/>
         <v>3.0952218555315892E-5</v>
       </c>
-      <c r="S23" s="15">
+      <c r="S23" s="14">
         <f t="shared" si="27"/>
         <v>1.2930009602971951E-2</v>
       </c>
       <c r="V23" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="W23" s="15">
+      <c r="W23" s="14">
         <f>STDEV(W18:W21)</f>
         <v>1.7344176635765891E-2</v>
       </c>
-      <c r="X23" s="15">
+      <c r="X23" s="14">
         <f t="shared" ref="X23:AC23" si="29">STDEV(X18:X21)</f>
         <v>1.3835102033444837E-3</v>
       </c>
-      <c r="Y23" s="15">
+      <c r="Y23" s="14">
         <f t="shared" si="29"/>
         <v>5.3417849284342782E-2</v>
       </c>
-      <c r="Z23" s="15">
+      <c r="Z23" s="14">
         <f t="shared" si="29"/>
         <v>1.2196860836732406E-2</v>
       </c>
-      <c r="AA23" s="15">
+      <c r="AA23" s="14">
         <f t="shared" si="29"/>
         <v>4.5098263519162018E-2</v>
       </c>
-      <c r="AB23" s="15">
+      <c r="AB23" s="14">
         <f t="shared" si="29"/>
         <v>1.0450173372558751E-4</v>
       </c>
-      <c r="AC23" s="15">
+      <c r="AC23" s="14">
         <f t="shared" si="29"/>
         <v>4.1843240150905799E-2</v>
       </c>
@@ -2350,650 +2340,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3B8E0FA-5F5A-C14F-8D5D-4EA1A8B93975}">
-  <dimension ref="A2:I23"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="10.83203125" style="3"/>
-    <col min="2" max="2" width="12.33203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="16384" width="10.83203125" style="3"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" s="9" t="s">
-        <v>1</v>
-      </c>
-      <c r="E3" s="9" t="s">
-        <v>2</v>
-      </c>
-      <c r="F3" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="G3" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="H3" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="I3" s="9" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A4" s="13" t="s">
-        <v>0</v>
-      </c>
-      <c r="B4" s="5">
-        <v>0</v>
-      </c>
-      <c r="C4" s="2">
-        <v>0.98510264087513499</v>
-      </c>
-      <c r="D4" s="2">
-        <v>0.10133650285281</v>
-      </c>
-      <c r="E4" s="2">
-        <v>0.89658234877307996</v>
-      </c>
-      <c r="F4" s="2">
-        <v>9.3382657181295108E-3</v>
-      </c>
-      <c r="G4" s="2">
-        <v>0.381381303081815</v>
-      </c>
-      <c r="H4" s="2">
-        <v>2.9177536106412302E-3</v>
-      </c>
-      <c r="I4" s="2">
-        <v>0.70680641611085004</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A5" s="13"/>
-      <c r="B5" s="7">
-        <v>0.5</v>
-      </c>
-      <c r="C5" s="8">
-        <v>0.990265018976482</v>
-      </c>
-      <c r="D5" s="8">
-        <v>0.10230459162844401</v>
-      </c>
-      <c r="E5" s="8">
-        <v>0.90490006398464395</v>
-      </c>
-      <c r="F5" s="8">
-        <v>5.6479140082498804E-3</v>
-      </c>
-      <c r="G5" s="8">
-        <v>0.455277690055649</v>
-      </c>
-      <c r="H5" s="8">
-        <v>2.4334868264778899E-3</v>
-      </c>
-      <c r="I5" s="8">
-        <v>0.62388016412893099</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A6" s="13"/>
-      <c r="B6" s="5">
-        <v>1</v>
-      </c>
-      <c r="C6" s="2">
-        <v>0.98057441213739605</v>
-      </c>
-      <c r="D6" s="2">
-        <v>9.2674994400380795E-2</v>
-      </c>
-      <c r="E6" s="2">
-        <v>0.85671541523666805</v>
-      </c>
-      <c r="F6" s="2">
-        <v>1.6463367569089098E-2</v>
-      </c>
-      <c r="G6" s="2">
-        <v>0.36921892846093102</v>
-      </c>
-      <c r="H6" s="2">
-        <v>3.2348737613528199E-3</v>
-      </c>
-      <c r="I6" s="2">
-        <v>0.71771453304142596</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A7" s="13"/>
-      <c r="B7" s="7">
-        <v>1.5</v>
-      </c>
-      <c r="C7" s="8">
-        <v>0.98307066176578295</v>
-      </c>
-      <c r="D7" s="8">
-        <v>9.6846614476140402E-2</v>
-      </c>
-      <c r="E7" s="8">
-        <v>0.89206259897153095</v>
-      </c>
-      <c r="F7" s="8">
-        <v>9.9562096405172405E-3</v>
-      </c>
-      <c r="G7" s="8">
-        <v>0.394857764169735</v>
-      </c>
-      <c r="H7" s="8">
-        <v>2.7749175470592599E-3</v>
-      </c>
-      <c r="I7" s="8">
-        <v>0.68905731777364698</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B8" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C8" s="12">
-        <f t="shared" ref="C8:I8" si="0">AVERAGE(C4:C7)</f>
-        <v>0.98475318343869911</v>
-      </c>
-      <c r="D8" s="12">
-        <f t="shared" si="0"/>
-        <v>9.82906758394438E-2</v>
-      </c>
-      <c r="E8" s="12">
-        <f t="shared" si="0"/>
-        <v>0.8875651067414807</v>
-      </c>
-      <c r="F8" s="12">
-        <f t="shared" si="0"/>
-        <v>1.0351439233996434E-2</v>
-      </c>
-      <c r="G8" s="12">
-        <f t="shared" si="0"/>
-        <v>0.40018392144203252</v>
-      </c>
-      <c r="H8" s="12">
-        <f t="shared" si="0"/>
-        <v>2.8402579363828E-3</v>
-      </c>
-      <c r="I8" s="12">
-        <f t="shared" si="0"/>
-        <v>0.68436460776371355</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B9" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C9" s="12">
-        <f>STDEV(C4:C7)</f>
-        <v>4.1148292902571095E-3</v>
-      </c>
-      <c r="D9" s="12">
-        <f t="shared" ref="D9:I9" si="1">STDEV(D4:D7)</f>
-        <v>4.4350788569674383E-3</v>
-      </c>
-      <c r="E9" s="12">
-        <f t="shared" si="1"/>
-        <v>2.1242585363527126E-2</v>
-      </c>
-      <c r="F9" s="12">
-        <f t="shared" si="1"/>
-        <v>4.4967226779570098E-3</v>
-      </c>
-      <c r="G9" s="12">
-        <f t="shared" si="1"/>
-        <v>3.8192759081880141E-2</v>
-      </c>
-      <c r="H9" s="12">
-        <f t="shared" si="1"/>
-        <v>3.3239501158298704E-4</v>
-      </c>
-      <c r="I9" s="12">
-        <f t="shared" si="1"/>
-        <v>4.2016828878300355E-2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A10" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="C10" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D10" s="9" t="s">
-        <v>1</v>
-      </c>
-      <c r="E10" s="9" t="s">
-        <v>2</v>
-      </c>
-      <c r="F10" s="9"/>
-      <c r="G10" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="H10" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="I10" s="9" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A11" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B11" s="5">
-        <v>0</v>
-      </c>
-      <c r="C11" s="4">
-        <v>0.96296666094613603</v>
-      </c>
-      <c r="D11" s="4">
-        <v>4.2715532785011799E-2</v>
-      </c>
-      <c r="E11" s="4">
-        <v>0.78663262544200296</v>
-      </c>
-      <c r="F11" s="4">
-        <v>1.5337397362387499E-2</v>
-      </c>
-      <c r="G11" s="4">
-        <v>0.56614912588484001</v>
-      </c>
-      <c r="H11" s="4">
-        <v>1.12898898125252E-3</v>
-      </c>
-      <c r="I11" s="4">
-        <v>0.33164503346349899</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A12" s="1"/>
-      <c r="B12" s="7">
-        <v>0.5</v>
-      </c>
-      <c r="C12" s="10">
-        <v>0.97367162815370301</v>
-      </c>
-      <c r="D12" s="10">
-        <v>4.3280663242661201E-2</v>
-      </c>
-      <c r="E12" s="10">
-        <v>0.78732496363780102</v>
-      </c>
-      <c r="F12" s="10">
-        <v>1.3587786605004E-3</v>
-      </c>
-      <c r="G12" s="10">
-        <v>0.48085685389592703</v>
-      </c>
-      <c r="H12" s="10">
-        <v>1.4075585068879901E-3</v>
-      </c>
-      <c r="I12" s="10">
-        <v>0.42627731384818301</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A13" s="1"/>
-      <c r="B13" s="5">
-        <v>1</v>
-      </c>
-      <c r="C13" s="6">
-        <v>0.97308473665731399</v>
-      </c>
-      <c r="D13" s="6">
-        <v>4.1375603007474997E-2</v>
-      </c>
-      <c r="E13" s="6">
-        <v>0.78992545327913999</v>
-      </c>
-      <c r="F13" s="6">
-        <v>3.2294661264048997E-5</v>
-      </c>
-      <c r="G13" s="6">
-        <v>0.48254989725200897</v>
-      </c>
-      <c r="H13" s="6">
-        <v>1.3471529262278101E-3</v>
-      </c>
-      <c r="I13" s="6">
-        <v>0.41669802466059502</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A14" s="1"/>
-      <c r="B14" s="7">
-        <v>1.5</v>
-      </c>
-      <c r="C14" s="10">
-        <v>0.94490458921929998</v>
-      </c>
-      <c r="D14" s="10">
-        <v>4.97667740138652E-2</v>
-      </c>
-      <c r="E14" s="10">
-        <v>0.72123666109484696</v>
-      </c>
-      <c r="F14" s="10">
-        <v>2.9937227655072202E-2</v>
-      </c>
-      <c r="G14" s="10">
-        <v>0.43733270461461698</v>
-      </c>
-      <c r="H14" s="10">
-        <v>2.1869368339852801E-3</v>
-      </c>
-      <c r="I14" s="10">
-        <v>0.57028474815171704</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B15" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C15" s="12">
-        <f t="shared" ref="C15:I15" si="2">AVERAGE(C11:C14)</f>
-        <v>0.96365690374411317</v>
-      </c>
-      <c r="D15" s="12">
-        <f t="shared" si="2"/>
-        <v>4.4284643262253301E-2</v>
-      </c>
-      <c r="E15" s="12">
-        <f t="shared" si="2"/>
-        <v>0.77127992586344785</v>
-      </c>
-      <c r="F15" s="12">
-        <f t="shared" si="2"/>
-        <v>1.1666424584806039E-2</v>
-      </c>
-      <c r="G15" s="12">
-        <f t="shared" si="2"/>
-        <v>0.49172214541184828</v>
-      </c>
-      <c r="H15" s="12">
-        <f t="shared" si="2"/>
-        <v>1.5176593120884E-3</v>
-      </c>
-      <c r="I15" s="12">
-        <f t="shared" si="2"/>
-        <v>0.4362262800309985</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B16" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C16" s="12">
-        <f>STDEV(C11:C14)</f>
-        <v>1.3432603043800383E-2</v>
-      </c>
-      <c r="D16" s="12">
-        <f t="shared" ref="D16:I16" si="3">STDEV(D11:D14)</f>
-        <v>3.7410496009907287E-3</v>
-      </c>
-      <c r="E16" s="12">
-        <f t="shared" si="3"/>
-        <v>3.339227786399826E-2</v>
-      </c>
-      <c r="F16" s="12">
-        <f t="shared" si="3"/>
-        <v>1.4010696265650055E-2</v>
-      </c>
-      <c r="G16" s="12">
-        <f t="shared" si="3"/>
-        <v>5.3850940532158602E-2</v>
-      </c>
-      <c r="H16" s="12">
-        <f t="shared" si="3"/>
-        <v>4.6194936313897729E-4</v>
-      </c>
-      <c r="I16" s="12">
-        <f t="shared" si="3"/>
-        <v>9.8976840210903888E-2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A17" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B17" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="C17" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D17" s="9" t="s">
-        <v>1</v>
-      </c>
-      <c r="E17" s="9" t="s">
-        <v>2</v>
-      </c>
-      <c r="F17" s="9"/>
-      <c r="G17" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="H17" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="I17" s="9" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A18" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="B18" s="5">
-        <v>0</v>
-      </c>
-      <c r="C18" s="4">
-        <v>0.92824506268345197</v>
-      </c>
-      <c r="D18" s="4">
-        <v>2.7065854937069901E-2</v>
-      </c>
-      <c r="E18" s="4">
-        <v>0.60608246195365401</v>
-      </c>
-      <c r="F18" s="4">
-        <v>2.4425167427614002E-3</v>
-      </c>
-      <c r="G18" s="4">
-        <v>0.682038516621988</v>
-      </c>
-      <c r="H18" s="4">
-        <v>7.7233959455626298E-4</v>
-      </c>
-      <c r="I18" s="4">
-        <v>0.24651273877889099</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A19" s="13"/>
-      <c r="B19" s="7">
-        <v>0.5</v>
-      </c>
-      <c r="C19" s="11">
-        <v>0.93970722578143695</v>
-      </c>
-      <c r="D19" s="11">
-        <v>2.4505204299938702E-2</v>
-      </c>
-      <c r="E19" s="11">
-        <v>0.62784426703959495</v>
-      </c>
-      <c r="F19" s="11">
-        <v>1.18808997260025E-4</v>
-      </c>
-      <c r="G19" s="11">
-        <v>0.67603131644803705</v>
-      </c>
-      <c r="H19" s="11">
-        <v>6.2081220557635498E-4</v>
-      </c>
-      <c r="I19" s="11">
-        <v>0.18062713171456601</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A20" s="13"/>
-      <c r="B20" s="5">
-        <v>1</v>
-      </c>
-      <c r="C20" s="4">
-        <v>0.92594645048404001</v>
-      </c>
-      <c r="D20" s="4">
-        <v>2.3943569866710201E-2</v>
-      </c>
-      <c r="E20" s="4">
-        <v>0.59994707479221598</v>
-      </c>
-      <c r="F20" s="4">
-        <v>1.59556026667219E-3</v>
-      </c>
-      <c r="G20" s="4">
-        <v>0.59789346306554203</v>
-      </c>
-      <c r="H20" s="4">
-        <v>8.6564896693274601E-4</v>
-      </c>
-      <c r="I20" s="4">
-        <v>0.274799156784302</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A21" s="13"/>
-      <c r="B21" s="7">
-        <v>1.5</v>
-      </c>
-      <c r="C21" s="11">
-        <v>0.89876678982603897</v>
-      </c>
-      <c r="D21" s="11">
-        <v>2.4652623061207201E-2</v>
-      </c>
-      <c r="E21" s="11">
-        <v>0.50717226095841605</v>
-      </c>
-      <c r="F21" s="11">
-        <v>2.5703641939036601E-2</v>
-      </c>
-      <c r="G21" s="11">
-        <v>0.69951637537677103</v>
-      </c>
-      <c r="H21" s="11">
-        <v>8.0739369825183504E-4</v>
-      </c>
-      <c r="I21" s="11">
-        <v>0.20610451158920601</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B22" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C22" s="12">
-        <f t="shared" ref="C22:I22" si="4">AVERAGE(C18:C21)</f>
-        <v>0.92316638219374203</v>
-      </c>
-      <c r="D22" s="12">
-        <f t="shared" si="4"/>
-        <v>2.5041813041231504E-2</v>
-      </c>
-      <c r="E22" s="12">
-        <f t="shared" si="4"/>
-        <v>0.58526151618597022</v>
-      </c>
-      <c r="F22" s="12">
-        <f t="shared" si="4"/>
-        <v>7.4651319864325544E-3</v>
-      </c>
-      <c r="G22" s="12">
-        <f t="shared" si="4"/>
-        <v>0.66386991787808447</v>
-      </c>
-      <c r="H22" s="12">
-        <f t="shared" si="4"/>
-        <v>7.665486163292998E-4</v>
-      </c>
-      <c r="I22" s="12">
-        <f t="shared" si="4"/>
-        <v>0.22701088471674125</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B23" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C23" s="12">
-        <f>STDEV(C18:C21)</f>
-        <v>1.7344176635765891E-2</v>
-      </c>
-      <c r="D23" s="12">
-        <f t="shared" ref="D23:I23" si="5">STDEV(D18:D21)</f>
-        <v>1.3835102033444837E-3</v>
-      </c>
-      <c r="E23" s="12">
-        <f t="shared" si="5"/>
-        <v>5.3417849284342782E-2</v>
-      </c>
-      <c r="F23" s="12">
-        <f t="shared" si="5"/>
-        <v>1.2196860836732406E-2</v>
-      </c>
-      <c r="G23" s="12">
-        <f t="shared" si="5"/>
-        <v>4.5098263519162018E-2</v>
-      </c>
-      <c r="H23" s="12">
-        <f t="shared" si="5"/>
-        <v>1.0450173372558751E-4</v>
-      </c>
-      <c r="I23" s="12">
-        <f t="shared" si="5"/>
-        <v>4.1843240150905799E-2</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A18:A21"/>
-    <mergeCell ref="A4:A7"/>
-    <mergeCell ref="A2:I2"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{22177130-642f-41d9-9211-74237ad5687d}" enabled="0" method="" siteId="{22177130-642f-41d9-9211-74237ad5687d}" removed="1"/>

</xml_diff>